<commit_message>
Fix cabinet overlapping in shop drawings, update DXF styling, and fix PDF scaling
</commit_message>
<xml_diff>
--- a/Albert_Project/outputs/23-033/23-033_Cabinet_Estimation.xlsx
+++ b/Albert_Project/outputs/23-033/23-033_Cabinet_Estimation.xlsx
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>378</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13">
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>127495.8376888889</v>
+        <v>80907.52376068378</v>
       </c>
     </row>
     <row r="14">
@@ -840,16 +840,16 @@
         <v>14</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="11" t="n">
         <v>0</v>
@@ -859,13 +859,13 @@
         <v/>
       </c>
       <c r="I5" s="11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5" s="12">
         <f>SUM(I5:K5)</f>
@@ -886,13 +886,13 @@
         <v>3</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>0</v>
@@ -905,13 +905,13 @@
         <v/>
       </c>
       <c r="I6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" s="12">
         <f>SUM(I6:K6)</f>
@@ -932,13 +932,13 @@
         <v>2</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>0</v>
@@ -951,13 +951,13 @@
         <v/>
       </c>
       <c r="I7" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" s="12">
         <f>SUM(I7:K7)</f>
@@ -978,13 +978,13 @@
         <v>3</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="11" t="n">
         <v>0</v>
@@ -997,13 +997,13 @@
         <v/>
       </c>
       <c r="I8" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="12">
         <f>SUM(I8:K8)</f>
@@ -1024,13 +1024,13 @@
         <v>3</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>0</v>
@@ -1043,13 +1043,13 @@
         <v/>
       </c>
       <c r="I9" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="11" t="n">
         <v>0</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L9" s="12">
         <f>SUM(I9:K9)</f>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>378</v>
+        <v>225</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E9" s="18" t="n">
-        <v>28659.806</v>
+        <v>15799.55</v>
       </c>
     </row>
     <row r="11">
@@ -2351,7 +2351,7 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>28659.806</v>
+        <v>15799.55</v>
       </c>
     </row>
     <row r="14">
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="E14" s="24" t="n">
-        <v>2149.48545</v>
+        <v>1184.96625</v>
       </c>
     </row>
     <row r="15">
@@ -2431,11 +2431,11 @@
       <c r="C17" s="22" t="n"/>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>$85/cabinet × 378 cabs</t>
+          <t>$85/cabinet × 225 cabs</t>
         </is>
       </c>
       <c r="E17" s="24" t="n">
-        <v>32130</v>
+        <v>19125</v>
       </c>
     </row>
     <row r="18">
@@ -2456,7 +2456,7 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>573.1961200000001</v>
+        <v>315.991</v>
       </c>
     </row>
     <row r="19">
@@ -2477,7 +2477,7 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>143.29903</v>
+        <v>78.99775000000001</v>
       </c>
     </row>
     <row r="20">
@@ -2498,7 +2498,7 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>229.278448</v>
+        <v>126.3964</v>
       </c>
     </row>
     <row r="21">
@@ -2532,7 +2532,7 @@
       <c r="C22" s="25" t="n"/>
       <c r="D22" s="25" t="n"/>
       <c r="E22" s="26" t="n">
-        <v>74585.06504799999</v>
+        <v>47330.9014</v>
       </c>
     </row>
     <row r="24">
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="E25" s="27" t="n">
-        <v>6374.791884444444</v>
+        <v>4045.376188034189</v>
       </c>
     </row>
     <row r="26">
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="E26" s="27" t="n">
-        <v>1912.437565333333</v>
+        <v>1213.612856410257</v>
       </c>
     </row>
     <row r="27">
@@ -2602,7 +2602,7 @@
         </is>
       </c>
       <c r="E27" s="27" t="n">
-        <v>44623.5431911111</v>
+        <v>28317.63331623932</v>
       </c>
     </row>
     <row r="30">
@@ -2612,7 +2612,7 @@
         </is>
       </c>
       <c r="E30" s="29" t="n">
-        <v>127495.8376888889</v>
+        <v>80907.52376068378</v>
       </c>
     </row>
     <row r="32">
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="E33" s="30" t="n">
-        <v>44623.5431911111</v>
+        <v>28317.63331623932</v>
       </c>
     </row>
     <row r="34">
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="E35" s="30" t="n">
-        <v>82872.29449777777</v>
+        <v>52589.89044444446</v>
       </c>
     </row>
     <row r="36">
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="E36" s="30" t="n">
-        <v>219.2388743327454</v>
+        <v>233.7328464197531</v>
       </c>
     </row>
     <row r="37">
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="E37" s="30" t="n">
-        <v>337.2905758965314</v>
+        <v>359.5889944919279</v>
       </c>
     </row>
   </sheetData>
@@ -2683,18 +2683,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="32" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2865,39 +2865,39 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>B30</t>
+          <t>W35-30</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>base 30.0"W × 28.3"H</t>
+          <t>upper_wall 35.4"W × 30.0"H</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>Base</t>
+          <t>Upper Wall</t>
         </is>
       </c>
       <c r="E11" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F11" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="F11" s="17" t="n">
-        <v>28.3</v>
-      </c>
       <c r="G11" s="17" t="n">
-        <v>23.6</v>
+        <v>13</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
-          <t>KITCHEN</t>
+          <t>UNIT A1 KITCHEN EL.</t>
         </is>
       </c>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>Kitchen, left of sink</t>
+          <t>Left of microwave shelf, top r</t>
         </is>
       </c>
     </row>
@@ -2907,39 +2907,39 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>SB35</t>
+          <t>MW30-15</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>sink_base 35.4"W × 28.3"H</t>
+          <t>microwave_shelf 30.0"W × 15.0"H</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>Sink Base</t>
+          <t>Microwave Shelf</t>
         </is>
       </c>
       <c r="E12" s="17" t="n">
-        <v>35.4</v>
+        <v>30</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>28.3</v>
+        <v>15</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>23.6</v>
+        <v>13</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>KITCHEN</t>
+          <t>UNIT A1 KITCHEN EL.</t>
         </is>
       </c>
       <c r="J12" s="16" t="inlineStr">
         <is>
-          <t>Kitchen, under sink</t>
+          <t>Above range, Elevation 1</t>
         </is>
       </c>
     </row>
@@ -2949,39 +2949,39 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>DWA24</t>
+          <t>W30-30</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>dw_adjacent 23.6"W × 28.3"H</t>
+          <t>upper_wall 30.0"W × 30.0"H</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>Dw Adjacent</t>
+          <t>Upper Wall</t>
         </is>
       </c>
       <c r="E13" s="17" t="n">
-        <v>23.6</v>
+        <v>30</v>
       </c>
       <c r="F13" s="17" t="n">
-        <v>28.3</v>
+        <v>30</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>23.6</v>
+        <v>13</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>KITCHEN</t>
+          <t>UNIT A1 KITCHEN EL.</t>
         </is>
       </c>
       <c r="J13" s="16" t="inlineStr">
         <is>
-          <t>Kitchen, right of sink</t>
+          <t xml:space="preserve">Right of microwave shelf, top </t>
         </is>
       </c>
     </row>
@@ -2991,39 +2991,39 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>W30-28</t>
+          <t>B35</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>upper_wall 30.0"W × 28.3"H</t>
+          <t>base 35.4"W × 28.3"H</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>Upper Wall</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="E14" s="17" t="n">
-        <v>30</v>
+        <v>35.4</v>
       </c>
       <c r="F14" s="17" t="n">
         <v>28.3</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>13</v>
+        <v>23.6</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>KITCHEN</t>
+          <t>UNIT A1 KITCHEN EL.</t>
         </is>
       </c>
       <c r="J14" s="16" t="inlineStr">
         <is>
-          <t>Kitchen, above left base cabin</t>
+          <t>Left of range, Elevation 1</t>
         </is>
       </c>
     </row>
@@ -3033,39 +3033,39 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>W35-28</t>
+          <t>B30</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>upper_wall 35.4"W × 28.3"H</t>
+          <t>base 30.0"W × 28.3"H</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>Upper Wall</t>
+          <t>Base</t>
         </is>
       </c>
       <c r="E15" s="17" t="n">
-        <v>35.4</v>
+        <v>30</v>
       </c>
       <c r="F15" s="17" t="n">
         <v>28.3</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>13</v>
+        <v>23.6</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>KITCHEN</t>
+          <t>UNIT A1 KITCHEN EL.</t>
         </is>
       </c>
       <c r="J15" s="16" t="inlineStr">
         <is>
-          <t>Kitchen, above sink</t>
+          <t>Right of range, Elevation 1</t>
         </is>
       </c>
     </row>
@@ -3075,39 +3075,39 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>W24-28</t>
+          <t>T12-84</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>upper_wall 23.6"W × 28.3"H</t>
+          <t>pantry 11.8"W × 83.9"H</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
-          <t>Upper Wall</t>
+          <t>Pantry</t>
         </is>
       </c>
       <c r="E16" s="17" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G16" s="17" t="n">
         <v>23.6</v>
       </c>
-      <c r="F16" s="17" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <v>13</v>
-      </c>
       <c r="H16" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I16" s="16" t="inlineStr">
         <is>
-          <t>KITCHEN</t>
+          <t>UNIT A1 KITCHEN EL.</t>
         </is>
       </c>
       <c r="J16" s="16" t="inlineStr">
         <is>
-          <t>Kitchen, above dishwasher spac</t>
+          <t>Right of refrigerator, Elevati</t>
         </is>
       </c>
     </row>
@@ -3117,24 +3117,24 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>MW30-15</t>
+          <t>W35-30</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>microwave_shelf 30.0"W × 15.0"H</t>
+          <t>upper_wall 35.4"W × 30.0"H</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
-          <t>Microwave Shelf</t>
+          <t>Upper Wall</t>
         </is>
       </c>
       <c r="E17" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F17" s="17" t="n">
         <v>30</v>
-      </c>
-      <c r="F17" s="17" t="n">
-        <v>15</v>
       </c>
       <c r="G17" s="17" t="n">
         <v>13</v>
@@ -3144,970 +3144,214 @@
       </c>
       <c r="I17" s="16" t="inlineStr">
         <is>
-          <t>KITCHEN</t>
+          <t>UNIT A1 KITCHEN EL.</t>
         </is>
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>Kitchen, above range</t>
+          <t>Left of refrigerator, Elevatio</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>SB35-ADA</t>
-        </is>
-      </c>
-      <c r="C18" s="16" t="inlineStr">
-        <is>
-          <t>sink_base 35.4"W × 34.0"H</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
-        <is>
-          <t>Sink Base</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="F18" s="17" t="n">
-        <v>34</v>
-      </c>
-      <c r="G18" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H18" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN PLAN</t>
-        </is>
-      </c>
-      <c r="J18" s="16" t="inlineStr">
-        <is>
-          <t>Kitchen, under sink</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>B18-ADA</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr">
-        <is>
-          <t>base 17.7"W × 34.0"H</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="n">
-        <v>17.7</v>
-      </c>
-      <c r="F19" s="17" t="n">
-        <v>34</v>
-      </c>
-      <c r="G19" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN PLAN</t>
-        </is>
-      </c>
-      <c r="J19" s="16" t="inlineStr">
-        <is>
-          <t>Kitchen, right of DW</t>
-        </is>
-      </c>
-    </row>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>KITCHEN SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="n"/>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
+    </row>
+    <row r="19"/>
     <row r="20">
-      <c r="A20" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>T24-84</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>pantry 23.6"W × 83.9"H</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>Pantry</t>
-        </is>
-      </c>
-      <c r="E20" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="F20" s="17" t="n">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="G20" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H20" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN PLAN</t>
-        </is>
-      </c>
-      <c r="J20" s="16" t="inlineStr">
-        <is>
-          <t>Kitchen, right of Refrigerator</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="n">
-        <v>11</v>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>T12-84</t>
-        </is>
-      </c>
-      <c r="C21" s="16" t="inlineStr">
-        <is>
-          <t>pantry 12.0"W × 83.9"H</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
-        <is>
-          <t>Pantry</t>
-        </is>
-      </c>
-      <c r="E21" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="F21" s="17" t="n">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="G21" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H21" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="16" t="inlineStr">
-        <is>
-          <t>General Notes</t>
-        </is>
-      </c>
-      <c r="J21" s="16" t="inlineStr">
-        <is>
-          <t>U9, General Notes</t>
-        </is>
-      </c>
-    </row>
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>SECTION 2 — BATHROOM VANITY CABINETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22">
-      <c r="A22" s="16" t="n">
-        <v>12</v>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>W35-30</t>
-        </is>
-      </c>
-      <c r="C22" s="16" t="inlineStr">
-        <is>
-          <t>upper_wall 35.4"W × 30.0"H</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
-        <is>
-          <t>Upper Wall</t>
-        </is>
-      </c>
-      <c r="E22" s="17" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="F22" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="G22" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="H22" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN EL.</t>
-        </is>
-      </c>
-      <c r="J22" s="16" t="inlineStr">
-        <is>
-          <t>Left of microwave shelf, top r</t>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Code</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>W (in)</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>H (in)</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>D (in)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Elev. Ref.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Location Note</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>MW30-15</t>
+          <t>VAN74</t>
         </is>
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>microwave_shelf 30.0"W × 15.0"H</t>
+          <t>vanity 74.0"W × 34.3"H</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
         <is>
-          <t>Microwave Shelf</t>
+          <t>Vanity</t>
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="F23" s="17" t="n">
-        <v>15</v>
+        <v>34.3</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>13</v>
+        <v>20.9</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>UNIT A1 KITCHEN EL.</t>
+          <t>A-6.00A</t>
         </is>
       </c>
       <c r="J23" s="16" t="inlineStr">
         <is>
-          <t>Above range, Elevation 1</t>
+          <t>Bathroom, left wall</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>W30-30</t>
+          <t>LIN24</t>
         </is>
       </c>
       <c r="C24" s="16" t="inlineStr">
         <is>
-          <t>upper_wall 30.0"W × 30.0"H</t>
+          <t>linen 23.6"W × 83.9"H</t>
         </is>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>Upper Wall</t>
+          <t>Linen</t>
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>30</v>
+        <v>23.6</v>
       </c>
       <c r="F24" s="17" t="n">
-        <v>30</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>13</v>
+        <v>23.6</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>1</v>
       </c>
       <c r="I24" s="16" t="inlineStr">
         <is>
-          <t>UNIT A1 KITCHEN EL.</t>
+          <t>A-6.00A</t>
         </is>
       </c>
       <c r="J24" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Right of microwave shelf, top </t>
+          <t>Bathroom, right of vanity</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>B35</t>
-        </is>
-      </c>
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>base 35.4"W × 28.3"H</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="E25" s="17" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="F25" s="17" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="G25" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H25" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I25" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN EL.</t>
-        </is>
-      </c>
-      <c r="J25" s="16" t="inlineStr">
-        <is>
-          <t>Left of range, Elevation 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>B30</t>
-        </is>
-      </c>
-      <c r="C26" s="16" t="inlineStr">
-        <is>
-          <t>base 30.0"W × 28.3"H</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="E26" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="F26" s="17" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="G26" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H26" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I26" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN EL.</t>
-        </is>
-      </c>
-      <c r="J26" s="16" t="inlineStr">
-        <is>
-          <t>Right of range, Elevation 1</t>
-        </is>
-      </c>
-    </row>
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>BATHROOM SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+    </row>
+    <row r="26"/>
     <row r="27">
-      <c r="A27" s="16" t="n">
-        <v>17</v>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>T12-84</t>
-        </is>
-      </c>
-      <c r="C27" s="16" t="inlineStr">
-        <is>
-          <t>pantry 11.8"W × 83.9"H</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr">
-        <is>
-          <t>Pantry</t>
-        </is>
-      </c>
-      <c r="E27" s="17" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="F27" s="17" t="n">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="G27" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H27" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN EL.</t>
-        </is>
-      </c>
-      <c r="J27" s="16" t="inlineStr">
-        <is>
-          <t>Right of refrigerator, Elevati</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="n">
-        <v>18</v>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>W35-30</t>
-        </is>
-      </c>
-      <c r="C28" s="16" t="inlineStr">
-        <is>
-          <t>upper_wall 35.4"W × 30.0"H</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
-        <is>
-          <t>Upper Wall</t>
-        </is>
-      </c>
-      <c r="E28" s="17" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="F28" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="G28" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="H28" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I28" s="16" t="inlineStr">
-        <is>
-          <t>UNIT A1 KITCHEN EL.</t>
-        </is>
-      </c>
-      <c r="J28" s="16" t="inlineStr">
-        <is>
-          <t>Left of refrigerator, Elevatio</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>KITCHEN SUBTOTALS</t>
-        </is>
-      </c>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
-      <c r="D29" s="25" t="n"/>
-      <c r="E29" s="25" t="n"/>
-      <c r="F29" s="25" t="n"/>
-      <c r="G29" s="25" t="n"/>
-      <c r="H29" s="13" t="n">
-        <v>18</v>
-      </c>
-      <c r="I29" s="25" t="n"/>
-      <c r="J29" s="25" t="n"/>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="32" t="inlineStr">
-        <is>
-          <t>SECTION 2 — BATHROOM VANITY CABINETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="9" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Cabinet Code</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>W (in)</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>H (in)</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>D (in)</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="I33" s="9" t="inlineStr">
-        <is>
-          <t>Elev. Ref.</t>
-        </is>
-      </c>
-      <c r="J33" s="9" t="inlineStr">
-        <is>
-          <t>Location Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>VAN74</t>
-        </is>
-      </c>
-      <c r="C34" s="16" t="inlineStr">
-        <is>
-          <t>vanity 74.0"W × 34.3"H</t>
-        </is>
-      </c>
-      <c r="D34" s="16" t="inlineStr">
-        <is>
-          <t>Vanity</t>
-        </is>
-      </c>
-      <c r="E34" s="17" t="n">
-        <v>74</v>
-      </c>
-      <c r="F34" s="17" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="G34" s="17" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="H34" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I34" s="16" t="inlineStr">
-        <is>
-          <t>A-6.00A</t>
-        </is>
-      </c>
-      <c r="J34" s="16" t="inlineStr">
-        <is>
-          <t>Bathroom, left wall</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>LIN24</t>
-        </is>
-      </c>
-      <c r="C35" s="16" t="inlineStr">
-        <is>
-          <t>linen 23.6"W × 83.9"H</t>
-        </is>
-      </c>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>Linen</t>
-        </is>
-      </c>
-      <c r="E35" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="F35" s="17" t="n">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="G35" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H35" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I35" s="16" t="inlineStr">
-        <is>
-          <t>A-6.00A</t>
-        </is>
-      </c>
-      <c r="J35" s="16" t="inlineStr">
-        <is>
-          <t>Bathroom, right of vanity</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>LIN24</t>
-        </is>
-      </c>
-      <c r="C36" s="16" t="inlineStr">
-        <is>
-          <t>linen 23.6"W × 83.9"H</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>Linen</t>
-        </is>
-      </c>
-      <c r="E36" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="F36" s="17" t="n">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="G36" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H36" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I36" s="16" t="inlineStr">
-        <is>
-          <t>BATHROOM</t>
-        </is>
-      </c>
-      <c r="J36" s="16" t="inlineStr">
-        <is>
-          <t>Bathroom, labeled 'LN.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>VAN35</t>
-        </is>
-      </c>
-      <c r="C37" s="16" t="inlineStr">
-        <is>
-          <t>vanity 35.4"W × 34.3"H</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>Vanity</t>
-        </is>
-      </c>
-      <c r="E37" s="17" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="F37" s="17" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="G37" s="17" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="H37" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I37" s="16" t="inlineStr">
-        <is>
-          <t>BATHROOM</t>
-        </is>
-      </c>
-      <c r="J37" s="16" t="inlineStr">
-        <is>
-          <t>Bathroom, under sink</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>VAN30</t>
-        </is>
-      </c>
-      <c r="C38" s="16" t="inlineStr">
-        <is>
-          <t>vanity 30.0"W × 34.3"H</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
-        <is>
-          <t>Vanity</t>
-        </is>
-      </c>
-      <c r="E38" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="F38" s="17" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="G38" s="17" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="H38" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I38" s="16" t="inlineStr">
-        <is>
-          <t>BATHROOM</t>
-        </is>
-      </c>
-      <c r="J38" s="16" t="inlineStr">
-        <is>
-          <t>Bathroom</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>LIN12</t>
-        </is>
-      </c>
-      <c r="C39" s="16" t="inlineStr">
-        <is>
-          <t>linen 12.0"W × 83.9"H</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>Linen</t>
-        </is>
-      </c>
-      <c r="E39" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="F39" s="17" t="n">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="G39" s="17" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="H39" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I39" s="16" t="inlineStr">
-        <is>
-          <t>General Notes</t>
-        </is>
-      </c>
-      <c r="J39" s="16" t="inlineStr">
-        <is>
-          <t>U14, General Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>VAN30-ADA</t>
-        </is>
-      </c>
-      <c r="C40" s="16" t="inlineStr">
-        <is>
-          <t>vanity 30.0"W × 34.3"H</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>Vanity</t>
-        </is>
-      </c>
-      <c r="E40" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="F40" s="17" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="G40" s="17" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="H40" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I40" s="16" t="inlineStr">
-        <is>
-          <t>General Notes</t>
-        </is>
-      </c>
-      <c r="J40" s="16" t="inlineStr">
-        <is>
-          <t>U20, General Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>MED30-ADA</t>
-        </is>
-      </c>
-      <c r="C41" s="16" t="inlineStr">
-        <is>
-          <t>medicine_cabinet 30.0"W × 28.3"H</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
-        <is>
-          <t>Medicine Cabinet</t>
-        </is>
-      </c>
-      <c r="E41" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="F41" s="17" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="G41" s="17" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="H41" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I41" s="16" t="inlineStr">
-        <is>
-          <t>General Notes</t>
-        </is>
-      </c>
-      <c r="J41" s="16" t="inlineStr">
-        <is>
-          <t>U8, General Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="16" t="n">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>UNIT A1 GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>VAN35</t>
-        </is>
-      </c>
-      <c r="C42" s="16" t="inlineStr">
-        <is>
-          <t>vanity 35.4"W × 34.3"H</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Vanity</t>
-        </is>
-      </c>
-      <c r="E42" s="17" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="F42" s="17" t="n">
-        <v>34.3</v>
-      </c>
-      <c r="G42" s="17" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="H42" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="16" t="inlineStr">
-        <is>
-          <t>ELEVATION_B</t>
-        </is>
-      </c>
-      <c r="J42" s="16" t="inlineStr">
-        <is>
-          <t>U20, FHA Bathroom Fixture Lege</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t>BATHROOM SUBTOTALS</t>
-        </is>
-      </c>
-      <c r="B43" s="25" t="n"/>
-      <c r="C43" s="25" t="n"/>
-      <c r="D43" s="25" t="n"/>
-      <c r="E43" s="25" t="n"/>
-      <c r="F43" s="25" t="n"/>
-      <c r="G43" s="25" t="n"/>
-      <c r="H43" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="I43" s="25" t="n"/>
-      <c r="J43" s="25" t="n"/>
-    </row>
-    <row r="44"/>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>UNIT A1 GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="n"/>
-      <c r="C45" s="25" t="n"/>
-      <c r="D45" s="25" t="n"/>
-      <c r="E45" s="25" t="n"/>
-      <c r="F45" s="25" t="n"/>
-      <c r="G45" s="25" t="n"/>
-      <c r="H45" s="33" t="n">
-        <v>27</v>
-      </c>
-      <c r="I45" s="25" t="n"/>
-      <c r="J45" s="25" t="n"/>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="25" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4120,8 +3364,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4137,6 +3393,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4222,6 +3479,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="32" t="inlineStr">
         <is>
@@ -4229,6 +3487,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -4282,11 +3541,498 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>No schedule available — PDF not processed</t>
-        </is>
-      </c>
+      <c r="A11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>W35-30-ADA</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Left of microwave shelf, top r</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>MW30-15-ADA</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>microwave_shelf 30.0"W × 15.0"H</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Microwave Shelf</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Above range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>W30-30-ADA</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 30.0"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Right of microwave shelf, top </t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>B35-ADA</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>base 35.4"W × 34.0"H</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Left of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>B30-ADA</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>base 30.0"W × 34.0"H</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Right of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>T12-84-ADA</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>pantry 11.8"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Pantry</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>Right of refrigerator, Elevati</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>W35-30-ADA</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Left of refrigerator, Elevatio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>KITCHEN SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="n"/>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>SECTION 2 — BATHROOM VANITY CABINETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Code</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>W (in)</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>H (in)</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>D (in)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Elev. Ref.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Location Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>VAN74-ADA</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>vanity 74.0"W × 34.0"H</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Vanity</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>74</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="G23" s="17" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, left wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>LIN24-ADA</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>linen 23.6"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Linen</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, right of vanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>BATHROOM SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>UNIT A2-ADA GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="25" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4299,8 +4045,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4316,6 +4074,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4401,6 +4160,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="32" t="inlineStr">
         <is>
@@ -4408,6 +4168,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -4461,11 +4222,498 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>No schedule available — PDF not processed</t>
-        </is>
-      </c>
+      <c r="A11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>W35-30</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Left of microwave shelf, top r</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>MW30-15</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>microwave_shelf 30.0"W × 15.0"H</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Microwave Shelf</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Above range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>W30-30</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 30.0"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Right of microwave shelf, top </t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>B35</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>base 35.4"W × 28.3"H</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Left of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>B30</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>base 30.0"W × 28.3"H</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Right of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>T12-84</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>pantry 11.8"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Pantry</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>Right of refrigerator, Elevati</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>W35-30</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Left of refrigerator, Elevatio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>KITCHEN SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="n"/>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>SECTION 2 — BATHROOM VANITY CABINETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Code</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>W (in)</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>H (in)</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>D (in)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Elev. Ref.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Location Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>VAN74</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>vanity 74.0"W × 34.3"H</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Vanity</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>74</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="G23" s="17" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, left wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>LIN24</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>linen 23.6"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Linen</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, right of vanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>BATHROOM SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>UNIT A3 GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="25" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4478,8 +4726,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4495,6 +4755,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4580,6 +4841,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="32" t="inlineStr">
         <is>
@@ -4587,6 +4849,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -4640,11 +4903,498 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>No schedule available — PDF not processed</t>
-        </is>
-      </c>
+      <c r="A11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>W35-30</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Left of microwave shelf, top r</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>MW30-15</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>microwave_shelf 30.0"W × 15.0"H</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Microwave Shelf</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Above range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>W30-30</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 30.0"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Right of microwave shelf, top </t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>B35</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>base 35.4"W × 28.3"H</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Left of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>B30</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>base 30.0"W × 28.3"H</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Right of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>T12-84</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>pantry 11.8"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Pantry</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>Right of refrigerator, Elevati</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>W35-30</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Left of refrigerator, Elevatio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>KITCHEN SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="n"/>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>SECTION 2 — BATHROOM VANITY CABINETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Code</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>W (in)</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>H (in)</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>D (in)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Elev. Ref.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Location Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>VAN74</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>vanity 74.0"W × 34.3"H</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Vanity</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>74</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="G23" s="17" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, left wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>LIN24</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>linen 23.6"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Linen</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, right of vanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>BATHROOM SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>UNIT B1 GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="25" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4657,8 +5407,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4674,6 +5436,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4759,6 +5522,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="32" t="inlineStr">
         <is>
@@ -4766,6 +5530,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -4819,11 +5584,498 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>No schedule available — PDF not processed</t>
-        </is>
-      </c>
+      <c r="A11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>W35-30-ADA</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Left of microwave shelf, top r</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>MW30-15-ADA</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>microwave_shelf 30.0"W × 15.0"H</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Microwave Shelf</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Above range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>W30-30-ADA</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 30.0"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H13" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Right of microwave shelf, top </t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>B35-ADA</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>base 35.4"W × 34.0"H</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Left of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>B30-ADA</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>base 30.0"W × 34.0"H</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Right of range, Elevation 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>T12-84-ADA</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>pantry 11.8"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Pantry</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>Right of refrigerator, Elevati</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>W35-30-ADA</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>upper_wall 35.4"W × 30.0"H</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Upper Wall</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="H17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>UNIT A1 KITCHEN EL.</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Left of refrigerator, Elevatio</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>KITCHEN SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="n"/>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>SECTION 2 — BATHROOM VANITY CABINETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Cabinet Code</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>W (in)</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>H (in)</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>D (in)</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Elev. Ref.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>Location Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>VAN74-ADA</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>vanity 74.0"W × 34.0"H</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Vanity</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n">
+        <v>74</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>34</v>
+      </c>
+      <c r="G23" s="17" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="H23" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, left wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>LIN24-ADA</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>linen 23.6"W × 83.9"H</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Linen</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="G24" s="17" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>A-6.00A</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>Bathroom, right of vanity</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>BATHROOM SUBTOTALS</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>UNIT B2-ADA GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="I27" s="25" t="n"/>
+      <c r="J27" s="25" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix shop drawing scaling and elevation rendering clipping issue
</commit_message>
<xml_diff>
--- a/Albert_Project/outputs/23-033/23-033_Cabinet_Estimation.xlsx
+++ b/Albert_Project/outputs/23-033/23-033_Cabinet_Estimation.xlsx
@@ -2885,7 +2885,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>1</v>
@@ -2927,7 +2927,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>1</v>
@@ -2969,7 +2969,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>1</v>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>base 35.4"W × 28.3"H</t>
+          <t>base 35.4"W × 28.4"H</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -3008,10 +3008,10 @@
         <v>35.4</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>1</v>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>base 30.0"W × 28.3"H</t>
+          <t>base 30.0"W × 28.4"H</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -3050,10 +3050,10 @@
         <v>30</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>1</v>
@@ -3095,7 +3095,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>1</v>
@@ -3137,7 +3137,7 @@
         <v>30</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>1</v>
@@ -3243,7 +3243,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>vanity 74.0"W × 34.3"H</t>
+          <t>vanity 74.0"W × 34.2"H</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -3255,10 +3255,10 @@
         <v>74</v>
       </c>
       <c r="F23" s="17" t="n">
-        <v>34.3</v>
+        <v>34.2</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>20.9</v>
+        <v>0.8</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>1</v>
@@ -3300,7 +3300,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>1</v>
@@ -3566,7 +3566,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>1</v>
@@ -3608,7 +3608,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>1</v>
@@ -3650,7 +3650,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>1</v>
@@ -3692,7 +3692,7 @@
         <v>34</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>1</v>
@@ -3734,7 +3734,7 @@
         <v>34</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>1</v>
@@ -3776,7 +3776,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>1</v>
@@ -3818,7 +3818,7 @@
         <v>30</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>1</v>
@@ -3939,7 +3939,7 @@
         <v>34</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>20.9</v>
+        <v>0.8</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>1</v>
@@ -3981,7 +3981,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>1</v>
@@ -4247,7 +4247,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>1</v>
@@ -4289,7 +4289,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>1</v>
@@ -4331,7 +4331,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>1</v>
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>base 35.4"W × 28.3"H</t>
+          <t>base 35.4"W × 28.4"H</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -4370,10 +4370,10 @@
         <v>35.4</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>1</v>
@@ -4400,7 +4400,7 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>base 30.0"W × 28.3"H</t>
+          <t>base 30.0"W × 28.4"H</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -4412,10 +4412,10 @@
         <v>30</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>1</v>
@@ -4457,7 +4457,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>1</v>
@@ -4499,7 +4499,7 @@
         <v>30</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>1</v>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>vanity 74.0"W × 34.3"H</t>
+          <t>vanity 74.0"W × 34.2"H</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -4617,10 +4617,10 @@
         <v>74</v>
       </c>
       <c r="F23" s="17" t="n">
-        <v>34.3</v>
+        <v>34.2</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>20.9</v>
+        <v>0.8</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>1</v>
@@ -4662,7 +4662,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>1</v>
@@ -4928,7 +4928,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>1</v>
@@ -4970,7 +4970,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>1</v>
@@ -5012,7 +5012,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>1</v>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>base 35.4"W × 28.3"H</t>
+          <t>base 35.4"W × 28.4"H</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -5051,10 +5051,10 @@
         <v>35.4</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>1</v>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>base 30.0"W × 28.3"H</t>
+          <t>base 30.0"W × 28.4"H</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -5093,10 +5093,10 @@
         <v>30</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>28.3</v>
+        <v>28.4</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>1</v>
@@ -5138,7 +5138,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>1</v>
@@ -5180,7 +5180,7 @@
         <v>30</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>1</v>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="C23" s="16" t="inlineStr">
         <is>
-          <t>vanity 74.0"W × 34.3"H</t>
+          <t>vanity 74.0"W × 34.2"H</t>
         </is>
       </c>
       <c r="D23" s="16" t="inlineStr">
@@ -5298,10 +5298,10 @@
         <v>74</v>
       </c>
       <c r="F23" s="17" t="n">
-        <v>34.3</v>
+        <v>34.2</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>20.9</v>
+        <v>0.8</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>1</v>
@@ -5343,7 +5343,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>1</v>
@@ -5609,7 +5609,7 @@
         <v>30</v>
       </c>
       <c r="G11" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H11" s="17" t="n">
         <v>1</v>
@@ -5651,7 +5651,7 @@
         <v>15</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H12" s="17" t="n">
         <v>1</v>
@@ -5693,7 +5693,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H13" s="17" t="n">
         <v>1</v>
@@ -5735,7 +5735,7 @@
         <v>34</v>
       </c>
       <c r="G14" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H14" s="17" t="n">
         <v>1</v>
@@ -5777,7 +5777,7 @@
         <v>34</v>
       </c>
       <c r="G15" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H15" s="17" t="n">
         <v>1</v>
@@ -5819,7 +5819,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G16" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H16" s="17" t="n">
         <v>1</v>
@@ -5861,7 +5861,7 @@
         <v>30</v>
       </c>
       <c r="G17" s="17" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="H17" s="17" t="n">
         <v>1</v>
@@ -5982,7 +5982,7 @@
         <v>34</v>
       </c>
       <c r="G23" s="17" t="n">
-        <v>20.9</v>
+        <v>0.8</v>
       </c>
       <c r="H23" s="17" t="n">
         <v>1</v>
@@ -6024,7 +6024,7 @@
         <v>83.90000000000001</v>
       </c>
       <c r="G24" s="17" t="n">
-        <v>23.6</v>
+        <v>0.9</v>
       </c>
       <c r="H24" s="17" t="n">
         <v>1</v>

</xml_diff>